<commit_message>
Major update, July 2025
</commit_message>
<xml_diff>
--- a/tables/table-1.xlsx
+++ b/tables/table-1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\44797\Desktop\Repo\national-canal-cooling\tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08C25CBA-30BF-4CCF-A3E4-2BB05950B4BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7A7DDA8-9DC4-4627-B001-602FBC526CCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{D818E9DE-A5FC-456E-864C-483B24EA8605}"/>
+    <workbookView xWindow="11520" yWindow="0" windowWidth="11520" windowHeight="12360" xr2:uid="{D818E9DE-A5FC-456E-864C-483B24EA8605}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -84,76 +84,6 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">−1.56 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(−2.19, −1.01)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">−1.60 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(−2.24, −1.04)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">−1.26 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(−1.78, −0.80)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>−1.09</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (−1.54, −0.70)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>−0.81</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (−1.15, −0.53)</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t>Median (</t>
     </r>
     <r>
@@ -247,296 +177,366 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">0.70 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(0.44, 1.03)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">−0.09 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(−0.15, −0.04)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">0.13 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(0.06, 0.23)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">0.49 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(0.30, 0.74)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">0.93 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(0.59, 1.35)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1.23 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(0.78, 1.76)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1.39 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(0.88, 2.00)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>−1.06</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (−1.50, −0.68)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1.46 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(0.92, 2.13)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1.38 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(0.87, 1.97)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1.08 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(0.68, 1.55)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>0.35</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (0.21, 0.54)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">0.17 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(0.09, 0.30)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>−0.78</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (−1.10, −0.50)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>−1.13</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (−1.59, −0.73)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>−1.25</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (−1.74, −0.80)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>−1.01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (−1.51, −0.65)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>−0.97</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (−1.38, −0.62)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>−0.90</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (−1.28, −0.58)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>−0.52</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (−0.74, −0.33)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>−0.25</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (−0.37, −0.16)</t>
+      <t>−0.77</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (−1.04, −0.72)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>−0.35</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (−0.35, −0.29)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>−0.83</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (−1.14, −0.73)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">−1.19 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(−1.33, −1.13)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">−1.34 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(−1.70, −1.18)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">−1.29 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(−1.68, −1.15)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>−1.36</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (−2.05, −1.28)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>−1.20</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (−1.83, −1.08)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>−1.05</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (−1.54, −0.93)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>−0.73</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (−0.89, −0.66)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>−0.56</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (−0.70, −0.48)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>−0.18</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (−0.24, −0.15)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>−0.26</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (−0.31, −0.24)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">0.16 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(0.15, 0.18)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">0.06 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(0.04, 0.08)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">0.09 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(0.06, 0.11)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">0.15 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(0.14, 0.17)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">0.15 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(0.13, 0.18)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">0.19 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(0.16, 0.20)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">0.18 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(0.14, 0.21)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">0.19 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(0.13, 0.20)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>0.21 (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>0.17, 0.21)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">0.30 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(0.27, 0.31)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>0.25</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (0.21, 0.26)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">0.24 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(0.22, 0.29)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>0.04</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (0.004, 0.05)</t>
     </r>
   </si>
 </sst>
@@ -1001,12 +1001,12 @@
   <sheetData>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B2" s="11" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C3" s="12" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="D3" s="12"/>
     </row>
@@ -1018,7 +1018,7 @@
         <v>14</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
@@ -1026,10 +1026,10 @@
         <v>0</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="I5" s="2"/>
     </row>
@@ -1038,10 +1038,10 @@
         <v>1</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="I6" s="2"/>
     </row>
@@ -1050,10 +1050,10 @@
         <v>2</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="I7" s="2"/>
     </row>
@@ -1062,10 +1062,10 @@
         <v>3</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="I8" s="2"/>
     </row>
@@ -1074,10 +1074,10 @@
         <v>4</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="I9" s="2"/>
     </row>
@@ -1086,10 +1086,10 @@
         <v>5</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="I10" s="2"/>
     </row>
@@ -1098,10 +1098,10 @@
         <v>6</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="I11" s="2"/>
     </row>
@@ -1110,10 +1110,10 @@
         <v>7</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="I12" s="2"/>
     </row>
@@ -1122,10 +1122,10 @@
         <v>8</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="I13" s="2"/>
     </row>
@@ -1134,10 +1134,10 @@
         <v>9</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="I14" s="2"/>
     </row>
@@ -1147,10 +1147,10 @@
         <v>10</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="I15" s="2"/>
     </row>
@@ -1159,10 +1159,10 @@
         <v>11</v>
       </c>
       <c r="C16" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="D16" s="8" t="s">
         <v>42</v>
-      </c>
-      <c r="D16" s="8" t="s">
-        <v>35</v>
       </c>
       <c r="I16" s="2"/>
     </row>
@@ -1171,7 +1171,7 @@
         <v>12</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="D17" s="8" t="s">
         <v>43</v>

</xml_diff>

<commit_message>
Updates to read-me file
</commit_message>
<xml_diff>
--- a/tables/table-1.xlsx
+++ b/tables/table-1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\44797\Desktop\Repo\national-canal-cooling\tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB05A005-318D-4963-A460-B476C5F267A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DCD72B2-E934-4090-8A32-4CBB3C396A8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11520" yWindow="0" windowWidth="11520" windowHeight="12360" xr2:uid="{D818E9DE-A5FC-456E-864C-483B24EA8605}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D818E9DE-A5FC-456E-864C-483B24EA8605}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -80,9 +80,6 @@
     <t>Time period</t>
   </si>
   <si>
-    <t>Daytime ∆T (°C)</t>
-  </si>
-  <si>
     <r>
       <t>Median (</t>
     </r>
@@ -123,6 +120,370 @@
         <family val="2"/>
       </rPr>
       <t>75)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>−0.77</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (−1.04, −0.72)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>−0.35</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (−0.35, −0.29)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>−0.83</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (−1.14, −0.73)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">−1.19 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(−1.33, −1.13)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">−1.34 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(−1.70, −1.18)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">−1.29 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(−1.68, −1.15)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>−1.36</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (−2.05, −1.28)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>−1.20</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (−1.83, −1.08)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>−1.05</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (−1.54, −0.93)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>−0.73</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (−0.89, −0.66)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>−0.56</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (−0.70, −0.48)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>−0.18</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (−0.24, −0.15)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>−0.26</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (−0.31, −0.24)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">0.16 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(0.15, 0.18)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">0.06 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(0.04, 0.08)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">0.09 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(0.06, 0.11)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">0.15 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(0.14, 0.17)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">0.15 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(0.13, 0.18)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">0.19 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(0.16, 0.20)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">0.18 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(0.14, 0.21)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">0.19 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(0.13, 0.20)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>0.21 (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>0.17, 0.21)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">0.30 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(0.27, 0.31)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>0.25</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (0.21, 0.26)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">0.24 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(0.22, 0.29)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>0.04</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (0.004, 0.05)</t>
     </r>
   </si>
   <si>
@@ -138,7 +499,7 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">T </t>
+      <t xml:space="preserve">PT </t>
     </r>
     <r>
       <rPr>
@@ -173,370 +534,51 @@
     </r>
   </si>
   <si>
-    <t>Nighttime ∆T (°C)</t>
-  </si>
-  <si>
-    <r>
-      <t>−0.77</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (−1.04, −0.72)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>−0.35</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (−0.35, −0.29)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>−0.83</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (−1.14, −0.73)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">−1.19 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(−1.33, −1.13)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">−1.34 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(−1.70, −1.18)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">−1.29 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(−1.68, −1.15)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>−1.36</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (−2.05, −1.28)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>−1.20</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (−1.83, −1.08)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>−1.05</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (−1.54, −0.93)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>−0.73</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (−0.89, −0.66)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>−0.56</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (−0.70, −0.48)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>−0.18</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (−0.24, −0.15)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>−0.26</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (−0.31, −0.24)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">0.16 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(0.15, 0.18)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">0.06 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(0.04, 0.08)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">0.09 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(0.06, 0.11)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">0.15 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(0.14, 0.17)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">0.15 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(0.13, 0.18)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">0.19 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(0.16, 0.20)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">0.18 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(0.14, 0.21)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">0.19 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(0.13, 0.20)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>0.21 (</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>0.17, 0.21)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">0.30 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(0.27, 0.31)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>0.25</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (0.21, 0.26)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">0.24 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(0.22, 0.29)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>0.04</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (0.004, 0.05)</t>
+    <r>
+      <t>Daytime ∆</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>PT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (°C)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Nighttime ∆</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>PT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (°C)</t>
     </r>
   </si>
 </sst>
@@ -544,7 +586,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -592,6 +634,13 @@
     </font>
     <font>
       <b/>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
       <i/>
       <sz val="11"/>
       <color theme="1"/>
@@ -1001,12 +1050,12 @@
   <sheetData>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B2" s="11" t="s">
-        <v>16</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C3" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D3" s="12"/>
     </row>
@@ -1015,10 +1064,10 @@
         <v>13</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>17</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
@@ -1026,10 +1075,10 @@
         <v>0</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="I5" s="2"/>
     </row>
@@ -1038,10 +1087,10 @@
         <v>1</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="I6" s="2"/>
     </row>
@@ -1050,10 +1099,10 @@
         <v>2</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="I7" s="2"/>
     </row>
@@ -1062,10 +1111,10 @@
         <v>3</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="I8" s="2"/>
     </row>
@@ -1074,10 +1123,10 @@
         <v>4</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="I9" s="2"/>
     </row>
@@ -1086,10 +1135,10 @@
         <v>5</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="I10" s="2"/>
     </row>
@@ -1098,10 +1147,10 @@
         <v>6</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="I11" s="2"/>
     </row>
@@ -1110,10 +1159,10 @@
         <v>7</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="I12" s="2"/>
     </row>
@@ -1122,10 +1171,10 @@
         <v>8</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="I13" s="2"/>
     </row>
@@ -1134,10 +1183,10 @@
         <v>9</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="I14" s="2"/>
     </row>
@@ -1147,10 +1196,10 @@
         <v>10</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="I15" s="2"/>
     </row>
@@ -1159,10 +1208,10 @@
         <v>11</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="I16" s="2"/>
     </row>
@@ -1171,10 +1220,10 @@
         <v>12</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="I17" s="2"/>
     </row>

</xml_diff>